<commit_message>
Update manufacturer nine-unit template format
</commit_message>
<xml_diff>
--- a/assets/manufacturer-nine-unit-template.xlsx
+++ b/assets/manufacturer-nine-unit-template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13500" windowHeight="12255"/>
+    <workbookView windowHeight="15620" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="企业背景单元" sheetId="9" r:id="rId1"/>
@@ -14,8 +14,7 @@
     <sheet name="能力单元" sheetId="4" r:id="rId5"/>
     <sheet name="案例单元" sheetId="5" r:id="rId6"/>
     <sheet name="对比单元" sheetId="6" r:id="rId7"/>
-    <sheet name="风控单元" sheetId="7" r:id="rId8"/>
-    <sheet name="采购支持单元" sheetId="8" r:id="rId9"/>
+    <sheet name="采购支持单元" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="125">
   <si>
     <t>公司名</t>
   </si>
@@ -77,6 +76,9 @@
   </si>
   <si>
     <t>WhatsApp</t>
+  </si>
+  <si>
+    <t>LINE</t>
   </si>
   <si>
     <t>邮箱</t>
@@ -137,15 +139,15 @@
     <t>参数</t>
   </si>
   <si>
-    <t>范围</t>
-  </si>
-  <si>
     <t>材质</t>
   </si>
   <si>
     <t>适用行业</t>
   </si>
   <si>
+    <t>产品卖点</t>
+  </si>
+  <si>
     <t>centrifugal fan</t>
   </si>
   <si>
@@ -158,9 +160,6 @@
     <t>7.5-75kW</t>
   </si>
   <si>
-    <t>0.6-1.0MPa</t>
-  </si>
-  <si>
     <t>Carbon Steel</t>
   </si>
   <si>
@@ -197,6 +196,9 @@
     <t>到期时间</t>
   </si>
   <si>
+    <t>适用产品</t>
+  </si>
+  <si>
     <t>ATEX</t>
   </si>
   <si>
@@ -230,9 +232,6 @@
     <t>工况</t>
   </si>
   <si>
-    <t>使用产品</t>
-  </si>
-  <si>
     <t>项目类型</t>
   </si>
   <si>
@@ -396,24 +395,6 @@
   </si>
   <si>
     <t>higher efficiency</t>
-  </si>
-  <si>
-    <t>风险类型</t>
-  </si>
-  <si>
-    <t>控制方式</t>
-  </si>
-  <si>
-    <t>企业措施</t>
-  </si>
-  <si>
-    <t>Overheating</t>
-  </si>
-  <si>
-    <t>Thermal protection</t>
-  </si>
-  <si>
-    <t>Temperature sensors</t>
   </si>
   <si>
     <t>交付方式</t>
@@ -1425,13 +1406,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultColWidth="24.6916666666667" defaultRowHeight="24" customHeight="1" outlineLevelRow="1"/>
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr defaultColWidth="24.6923076923077" defaultRowHeight="24" customHeight="1" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="16384" width="24.6916666666667" style="3" customWidth="1"/>
+    <col min="1" max="16384" width="24.6923076923077" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:15">
+    <row r="1" customHeight="1" spans="1:16">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1477,49 +1458,52 @@
       <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
+      <c r="P1" s="3" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" customHeight="1" spans="1:15">
+    <row r="2" customHeight="1" spans="1:16">
       <c r="A2" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2" s="3">
         <v>2009</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="O2" s="3" t="s">
         <v>27</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -1532,54 +1516,52 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultColWidth="24.6916666666667" defaultRowHeight="24" customHeight="1" outlineLevelRow="1" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="24.6923076923077" defaultRowHeight="24" customHeight="1" outlineLevelRow="1" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="16384" width="24.6916666666667" style="3" customWidth="1"/>
+    <col min="1" max="16383" width="24.6923076923077" style="3" customWidth="1"/>
+    <col min="16384" max="16384" width="24.6923076923077" style="3"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="1:7">
       <c r="A1" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:7">
       <c r="A2" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G2" s="3" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1592,15 +1574,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultColWidth="24.6916666666667" defaultRowHeight="24" customHeight="1" outlineLevelRow="1"/>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultColWidth="24.6923076923077" defaultRowHeight="24" customHeight="1" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="3" width="24.6916666666667" style="3" customWidth="1"/>
-    <col min="4" max="4" width="24.6916666666667" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="24.6916666666667" style="3" customWidth="1"/>
+    <col min="1" max="3" width="24.6923076923077" style="3" customWidth="1"/>
+    <col min="4" max="4" width="24.6923076923077" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="24.6923076923077" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:10">
+    <row r="1" customHeight="1" spans="1:11">
       <c r="A1" s="3" t="s">
         <v>42</v>
       </c>
@@ -1610,7 +1592,7 @@
       <c r="C1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>45</v>
       </c>
       <c r="E1" s="3" t="s">
@@ -1631,37 +1613,43 @@
       <c r="J1" s="3" t="s">
         <v>51</v>
       </c>
+      <c r="K1" s="3" t="s">
+        <v>52</v>
+      </c>
     </row>
-    <row r="2" customHeight="1" spans="1:10">
+    <row r="2" customHeight="1" spans="1:11">
       <c r="A2" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D2" s="4" t="s">
         <v>55</v>
       </c>
+      <c r="D2" s="3" t="s">
+        <v>56</v>
+      </c>
       <c r="E2" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I2" s="3">
         <v>45078</v>
       </c>
       <c r="J2" s="3">
         <v>46905</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -1674,25 +1662,25 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultColWidth="24.6916666666667" defaultRowHeight="24" customHeight="1" outlineLevelRow="1"/>
+  <sheetFormatPr defaultColWidth="24.6923076923077" defaultRowHeight="24" customHeight="1" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="3" width="24.6916666666667" style="3" customWidth="1"/>
-    <col min="4" max="4" width="24.6916666666667" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="24.6916666666667" style="3" customWidth="1"/>
+    <col min="1" max="3" width="24.6923076923077" style="3" customWidth="1"/>
+    <col min="4" max="4" width="24.6923076923077" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="24.6923076923077" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="1:9">
       <c r="A1" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1" s="4" t="s">
         <v>63</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>52</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>64</v>
@@ -1720,8 +1708,8 @@
       <c r="C2" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>36</v>
+      <c r="D2" s="3" t="s">
+        <v>37</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>71</v>
@@ -1749,9 +1737,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultColWidth="24.6916666666667" defaultRowHeight="24" customHeight="1" outlineLevelRow="1" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="24.6923076923077" defaultRowHeight="24" customHeight="1" outlineLevelRow="1" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="16384" width="24.6916666666667" style="3" customWidth="1"/>
+    <col min="1" max="16384" width="24.6923076923077" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="1:8">
@@ -1816,11 +1804,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultColWidth="24.6916666666667" defaultRowHeight="24" customHeight="1" outlineLevelRow="1" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="24.6923076923077" defaultRowHeight="24" customHeight="1" outlineLevelRow="1" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="3" width="24.6916666666667" style="3" customWidth="1"/>
-    <col min="4" max="4" width="24.6916666666667" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="24.6916666666667" style="3" customWidth="1"/>
+    <col min="1" max="3" width="24.6923076923077" style="3" customWidth="1"/>
+    <col min="4" max="4" width="24.6923076923077" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="24.6923076923077" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="1:8">
@@ -1828,12 +1816,12 @@
         <v>92</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>94</v>
       </c>
       <c r="E1" s="3" t="s">
@@ -1859,8 +1847,8 @@
       <c r="C2" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>36</v>
+      <c r="D2" s="3" t="s">
+        <v>37</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>101</v>
@@ -1885,11 +1873,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultColWidth="24.6916666666667" defaultRowHeight="24" customHeight="1" outlineLevelRow="1" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="24.6923076923077" defaultRowHeight="24" customHeight="1" outlineLevelRow="1" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="3" width="24.6916666666667" style="3" customWidth="1"/>
-    <col min="4" max="4" width="24.6916666666667" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="24.6916666666667" style="3" customWidth="1"/>
+    <col min="1" max="3" width="24.6923076923077" style="3" customWidth="1"/>
+    <col min="4" max="4" width="24.6923076923077" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="24.6923076923077" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customHeight="1" spans="1:7">
@@ -1902,7 +1890,7 @@
       <c r="C1" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>108</v>
       </c>
       <c r="E1" s="3" t="s">
@@ -1925,7 +1913,7 @@
       <c r="C2" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>115</v>
       </c>
       <c r="E2" s="3" t="s">
@@ -1947,75 +1935,44 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="24.6916666666667" defaultRowHeight="24" customHeight="1" outlineLevelRow="1" outlineLevelCol="2"/>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultColWidth="24.6923076923077" defaultRowHeight="24" customHeight="1" outlineLevelRow="1" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="16384" width="24.6916666666667" style="3" customWidth="1"/>
+    <col min="1" max="16384" width="24.6923076923077" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:3">
-      <c r="A1" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="2" customHeight="1" spans="1:3">
-      <c r="A2" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="24.6916666666667" defaultRowHeight="24" customHeight="1" outlineLevelRow="1" outlineLevelCol="3"/>
-  <cols>
-    <col min="1" max="16384" width="24.6916666666667" style="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" customHeight="1" spans="1:4">
+    <row r="1" customHeight="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>80</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>52</v>
       </c>
     </row>
-    <row r="2" customHeight="1" spans="1:4">
+    <row r="2" customHeight="1" spans="1:5">
       <c r="A2" s="1" t="s">
         <v>88</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>130</v>
+        <v>124</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>